<commit_message>
Nebenkosten 2025: Vorauszahlung bestaetigt
Die 3.600 EUR fuer 2025 sind bestaetigt, 300 EUR im Monat wie im Vorjahr.
Annahme-Markierung entfernt, damit ist die Abrechnung versandfertig:
Guthaben 1.594,49 EUR.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2Vxc1sWTkdQ9c9u5jSatw
</commit_message>
<xml_diff>
--- a/10_Output/2026-10-26-nebenkosten-2025-ingelheim-whg3-huber.xlsx
+++ b/10_Output/2026-10-26-nebenkosten-2025-ingelheim-whg3-huber.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Abrechnung!$A$1:$G$52</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">'Aus dem Protokoll'!$A$1:$B$12</definedName>
-    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">'Herkunft und Pruefung'!$A$1:$E$31</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">'Herkunft und Pruefung'!$A$1:$E$30</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -70,24 +70,12 @@
         </r>
       </text>
     </comment>
-    <comment ref="G35" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">ANNAHME: 300,00 € im Monat wie 2024. Vor dem Versenden gegen die tatsächlich eingegangenen Zahlungen prüfen und hier berichtigen — alles Weitere rechnet sich neu.</t>
-        </r>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="104">
   <si>
     <t xml:space="preserve">Sascha Coldewey</t>
   </si>
@@ -327,12 +315,6 @@
   </si>
   <si>
     <t xml:space="preserve">Vor dem Versenden</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vorauszahlungen 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Die 3.600 € sind aus 2024 übernommen. Gegen die tatsächlichen Eingänge auf deinem Konto prüfen und in der Abrechnung berichtigen.</t>
   </si>
   <si>
     <t xml:space="preserve">Abrechnungsfrist</t>
@@ -416,7 +398,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.000"/>
     <numFmt numFmtId="166" formatCode="#,##0.00&quot; €&quot;;\-#,##0.00&quot; €&quot;;\-"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -482,13 +464,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
       <b val="true"/>
       <sz val="12"/>
       <name val="Arial"/>
@@ -508,7 +483,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -531,12 +506,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
         <bgColor rgb="FFE8E8E8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF99"/>
-        <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -604,7 +573,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -677,23 +646,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1442,20 +1407,20 @@
       <c r="D35" s="6"/>
       <c r="E35" s="6"/>
       <c r="F35" s="6"/>
-      <c r="G35" s="18" t="n">
+      <c r="G35" s="14" t="n">
         <v>3600</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="19" t="s">
+      <c r="A36" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="B36" s="19"/>
-      <c r="C36" s="19"/>
-      <c r="D36" s="19"/>
-      <c r="E36" s="19"/>
-      <c r="F36" s="19"/>
-      <c r="G36" s="20" t="n">
+      <c r="B36" s="18"/>
+      <c r="C36" s="18"/>
+      <c r="D36" s="18"/>
+      <c r="E36" s="18"/>
+      <c r="F36" s="18"/>
+      <c r="G36" s="19" t="n">
         <f aca="false">G35-G34</f>
         <v>1594.49</v>
       </c>
@@ -1522,24 +1487,24 @@
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="21"/>
-      <c r="B51" s="21"/>
-      <c r="C51" s="21"/>
-      <c r="D51" s="21"/>
-      <c r="E51" s="21"/>
-      <c r="F51" s="21"/>
-      <c r="G51" s="21"/>
+      <c r="A51" s="20"/>
+      <c r="B51" s="20"/>
+      <c r="C51" s="20"/>
+      <c r="D51" s="20"/>
+      <c r="E51" s="20"/>
+      <c r="F51" s="20"/>
+      <c r="G51" s="20"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="22" t="s">
+      <c r="A52" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="B52" s="22"/>
-      <c r="C52" s="22"/>
-      <c r="D52" s="22"/>
-      <c r="E52" s="22"/>
-      <c r="F52" s="22"/>
-      <c r="G52" s="22"/>
+      <c r="B52" s="21"/>
+      <c r="C52" s="21"/>
+      <c r="D52" s="21"/>
+      <c r="E52" s="21"/>
+      <c r="F52" s="21"/>
+      <c r="G52" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="15">
@@ -1575,7 +1540,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -1585,12 +1550,12 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="22" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="23" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1606,7 +1571,7 @@
       <c r="C5" s="14" t="n">
         <v>1992.51</v>
       </c>
-      <c r="E5" s="25" t="s">
+      <c r="E5" s="24" t="s">
         <v>57</v>
       </c>
     </row>
@@ -1617,7 +1582,7 @@
       <c r="C6" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="E6" s="25" t="s">
+      <c r="E6" s="24" t="s">
         <v>59</v>
       </c>
     </row>
@@ -1625,10 +1590,10 @@
       <c r="A7" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C7" s="26" t="n">
+      <c r="C7" s="25" t="n">
         <v>2005.51</v>
       </c>
-      <c r="E7" s="25"/>
+      <c r="E7" s="24"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
@@ -1642,7 +1607,7 @@
       <c r="C10" s="14" t="n">
         <v>499.8</v>
       </c>
-      <c r="E10" s="27" t="s">
+      <c r="E10" s="26" t="s">
         <v>63</v>
       </c>
     </row>
@@ -1653,7 +1618,7 @@
       <c r="C11" s="14" t="n">
         <v>45.6</v>
       </c>
-      <c r="E11" s="27"/>
+      <c r="E11" s="26"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
@@ -1662,7 +1627,7 @@
       <c r="C12" s="14" t="n">
         <v>34.47</v>
       </c>
-      <c r="E12" s="27"/>
+      <c r="E12" s="26"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
@@ -1671,7 +1636,7 @@
       <c r="C13" s="14" t="n">
         <v>18.65</v>
       </c>
-      <c r="E13" s="27"/>
+      <c r="E13" s="26"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
@@ -1718,10 +1683,10 @@
       <c r="A20" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C20" s="28" t="s">
+      <c r="C20" s="27" t="s">
         <v>73</v>
       </c>
-      <c r="D20" s="28" t="s">
+      <c r="D20" s="27" t="s">
         <v>74</v>
       </c>
     </row>
@@ -1735,7 +1700,7 @@
       <c r="D21" s="14" t="n">
         <v>2005.51</v>
       </c>
-      <c r="E21" s="27" t="s">
+      <c r="E21" s="26" t="s">
         <v>76</v>
       </c>
     </row>
@@ -1749,7 +1714,7 @@
       <c r="D22" s="14" t="n">
         <v>1312.86</v>
       </c>
-      <c r="E22" s="27"/>
+      <c r="E22" s="26"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
@@ -1761,7 +1726,7 @@
       <c r="D23" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="E23" s="27"/>
+      <c r="E23" s="26"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
@@ -1769,7 +1734,7 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="29" t="s">
+      <c r="A26" s="28" t="s">
         <v>80</v>
       </c>
       <c r="B26" s="7" t="s">
@@ -1780,30 +1745,30 @@
       <c r="E26" s="7"/>
     </row>
     <row r="27" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="29" t="s">
+      <c r="A27" s="28" t="s">
+        <v>31</v>
+      </c>
+      <c r="B27" s="7" t="s">
         <v>82</v>
-      </c>
-      <c r="B27" s="7" t="s">
-        <v>83</v>
       </c>
       <c r="C27" s="7"/>
       <c r="D27" s="7"/>
       <c r="E27" s="7"/>
     </row>
     <row r="28" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="29" t="s">
-        <v>31</v>
+      <c r="A28" s="28" t="s">
+        <v>28</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C28" s="7"/>
       <c r="D28" s="7"/>
       <c r="E28" s="7"/>
     </row>
     <row r="29" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="29" t="s">
-        <v>28</v>
+      <c r="A29" s="28" t="s">
+        <v>84</v>
       </c>
       <c r="B29" s="7" t="s">
         <v>85</v>
@@ -1812,26 +1777,14 @@
       <c r="D29" s="7"/>
       <c r="E29" s="7"/>
     </row>
-    <row r="30" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="29" t="s">
-        <v>86</v>
-      </c>
-      <c r="B30" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="C30" s="7"/>
-      <c r="D30" s="7"/>
-      <c r="E30" s="7"/>
-    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="6">
     <mergeCell ref="E10:E13"/>
     <mergeCell ref="E21:E23"/>
     <mergeCell ref="B26:E26"/>
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="B28:E28"/>
     <mergeCell ref="B29:E29"/>
-    <mergeCell ref="B30:E30"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1856,77 +1809,77 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="22" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="23" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="28" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="24" t="s">
+      <c r="B4" s="29" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="29" t="s">
+    <row r="5" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="28" t="s">
         <v>90</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="B5" s="29" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="29" t="s">
+    <row r="6" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="B5" s="30" t="s">
+      <c r="B6" s="29" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="29" t="s">
+    <row r="7" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="28" t="s">
         <v>94</v>
       </c>
-      <c r="B6" s="30" t="s">
+      <c r="B7" s="29" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="29" t="s">
+    <row r="8" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="28" t="s">
         <v>96</v>
       </c>
-      <c r="B7" s="30" t="s">
+      <c r="B8" s="29" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="29" t="s">
+    <row r="9" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="28" t="s">
         <v>98</v>
       </c>
-      <c r="B8" s="30" t="s">
+      <c r="B9" s="29" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="29" t="s">
+    <row r="10" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="28" t="s">
         <v>100</v>
       </c>
-      <c r="B9" s="30" t="s">
+      <c r="B10" s="29" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="29" t="s">
+    <row r="11" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="28" t="s">
         <v>102</v>
       </c>
-      <c r="B10" s="30" t="s">
+      <c r="B11" s="29" t="s">
         <v>103</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="29" t="s">
-        <v>104</v>
-      </c>
-      <c r="B11" s="30" t="s">
-        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ingelheim: Vorauszahlung steht bereits auf 200 EUR
Die 840 EUR von Huber sind 640 EUR Kaltmiete plus 200 EUR Vorauszahlung.
Die Senkung von 300 EUR ist bereits erfolgt, fuer 2024 und 2025 galten noch
300 EUR - die Abrechnung 2025 bleibt richtig.

Der Absatz im Anschreiben, der eine Senkung auf 185 EUR vorschlug, ist durch
einen ersetzt, der die bestehenden 200 EUR bestaetigt und einordnet.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2Vxc1sWTkdQ9c9u5jSatw
</commit_message>
<xml_diff>
--- a/10_Output/2026-10-26-nebenkosten-2025-ingelheim-whg3-huber.xlsx
+++ b/10_Output/2026-10-26-nebenkosten-2025-ingelheim-whg3-huber.xlsx
@@ -65,8 +65,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">2.005,51 € im Jahr sind 167,13 € im Monat. 185 € lassen Luft für steigende Energiepreise. Die Herabsetzung ist nach § 560 Abs. 4 BGB zulässig und muss in Textform erklärt werden — dieser Absatz genügt dafür.
-Betrag frei wählbar.</t>
+          <t xml:space="preserve">2.005,51 € im Jahr sind 167,13 € im Monat, die Vorauszahlung liegt bei 200 € — das passt. Zusammen mit der Kaltmiete von 640 € ergibt das die 840 €, die Huber überweist.</t>
         </r>
       </text>
     </comment>
@@ -224,7 +223,7 @@
     <t xml:space="preserve">Das Guthaben überweise ich Ihnen innerhalb von 14 Tagen auf Ihr bekanntes Konto.</t>
   </si>
   <si>
-    <t xml:space="preserve">Anpassung der Vorauszahlung: Ihre monatliche Vorauszahlung liegt deutlich über den tatsächlichen Kosten. Ab dem nächsten Monat setze ich sie auf 185,00 € herab. Damit entsteht weder für Sie noch für mich eine größere Nachzahlung.</t>
+    <t xml:space="preserve">Zur Vorauszahlung: Ihre monatliche Vorauszahlung haben wir bereits von 300,00 € auf 200,00 € gesenkt. Gemessen an den Kosten des Jahres 2025 von 167,13 € im Monat bleibt damit ein angemessener Puffer für steigende Energiepreise. Eine weitere Änderung ist derzeit nicht vorgesehen.</t>
   </si>
   <si>
     <t xml:space="preserve">Die Bescheinigung über haushaltsnahe Dienstleistungen und Handwerkerleistungen nach § 35a EStG liegt bei. Sie können daraus 295,69 € und 175,43 € in Ihrer Einkommensteuererklärung geltend machen.</t>

</xml_diff>

<commit_message>
Ingelheim: Vorauszahlung belegt, Positionsvergleich, drei Absender
Auf Nachfrage geprueft: Der Mietvertrag nennt nur 200 EUR Vorauszahlung,
gezahlt wurden aber 300 EUR. Das ist vierfach belegt - eigene Abrechnung
2023, Verwaltungsabrechnung 2024, Zahlungshistorie und unveraenderte
Kaltmiete. Eine Erklaerung zur Erhoehung liegt nicht vor.

Positionsvergleich 2024 gegen 2025: insgesamt 214,27 EUR mehr umgelegt, bei
den kalten Betriebskosten 128,84 EUR weniger. Zwei der vier fehlenden
Positionen sind erklaert, bei Hebeanlage und Rauchwarnmeldern ist die Frage,
ob die Wartungen stattfanden.

Nebenbefund: Die Abrechnung 2023 kam von der Coldewey Holding GmbH, der
Mietvertrag nennt Elimar Coldewey, die Schreiben 2026 Sascha privat. Drei
Absender fuer ein Mietverhaeltnis, Eigentuemer ist durchgehend Sascha privat.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2Vxc1sWTkdQ9c9u5jSatw
</commit_message>
<xml_diff>
--- a/10_Output/2026-10-26-nebenkosten-2025-ingelheim-whg3-huber.xlsx
+++ b/10_Output/2026-10-26-nebenkosten-2025-ingelheim-whg3-huber.xlsx
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="118">
   <si>
     <t xml:space="preserve">Sascha Coldewey</t>
   </si>
@@ -292,7 +292,7 @@
     <t xml:space="preserve">Summe</t>
   </si>
   <si>
-    <t xml:space="preserve">Vergleich mit 2024</t>
+    <t xml:space="preserve">Jede Position im Vergleich mit 2024</t>
   </si>
   <si>
     <t xml:space="preserve">2024</t>
@@ -301,37 +301,83 @@
     <t xml:space="preserve">2025</t>
   </si>
   <si>
-    <t xml:space="preserve">Umlagefähige Kosten gesamt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plus 214,27 € oder 12 %. Der Anstieg kommt allein von Heizung und Wasser; Kabelfernsehen ist seit dem 01.07.2024 nicht mehr umlagefähig und 2025 zu Recht ganz entfallen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">davon Heizung, Wasser, Abwasser</t>
+    <t xml:space="preserve">Differenz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abrechnungsfrist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Für 2025 läuft sie am 31.12.2026 ab (§ 556 Abs. 3 BGB). Danach kannst du nichts mehr nachfordern. Da es ein Guthaben ist, droht dir kein Verlust — aber die Herabsetzung der Vorauszahlung willst du rechtzeitig wirksam machen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,55 € ohne nähere Bezeichnung. Beim Verwalter erfragen, was dahinter steckt — ein Mieter darf das wissen wollen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9,63 € sind umlagefähig (§ 2 Nr. 2 BetrKV). Nicht zu verwechseln mit der Miete von Rauchwarnmeldern, die es nicht wäre.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Belegeinsicht</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Du musst sie gewähren, wenn Huber darum bittet. Die Unterlagen der Verwaltung bereithalten.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">neu, § 2 Nr. 2 BetrKV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sonstige umlagefähig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">neu, Zweck unbekannt</t>
   </si>
   <si>
     <t xml:space="preserve">Kabelfernsehen</t>
   </si>
   <si>
+    <t xml:space="preserve">zu Recht entfallen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abrechnung Heiz-/Wasserkosten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">steckt jetzt in den Heizkosten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hebeanlage Wartung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRÜFEN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wartung Rauchmelder/Löscher</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summe kalte Betriebskosten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Heizung, Wasser, Abwasser</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gesamt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Antwort auf die Frage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insgesamt legst du 214,27 € MEHR um als 2024, nämlich 2.005,51 € statt 1.791,24 €. Bei den kalten Betriebskosten legst du dagegen 128,84 € WENIGER um. Der Unterschied kommt von vier Positionen, die 2025 fehlen:
+• Kabelfernsehen (93,96 €) ist seit dem 01.07.2024 nicht mehr umlagefähig und zu Recht entfallen. Kein Verlust.
+• Die Abrechnungskosten (37,24 €) stecken 2025 in den Heizkosten — die Heizkostenabrechnung weist dort 260,55 € Zusatzkosten aus, fast genau den Betrag, der 2024 separat stand. Nur umgezogen, nicht verloren.
+• Hebeanlage (52,70 €) und Rauchwarnmelder (8,73 €) fehlen ohne erkennbaren Grund. Zusammen 61,43 €.
+Bei den letzten beiden geht es weniger ums Geld als um die Frage, ob die Wartungen überhaupt stattgefunden haben. Rauchwarnmelder sind jährlich zu prüfen, und eine Abwasserhebeanlage will regelmäßig gewartet werden. Beim Verwalter nachfragen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Und der Heizkostenanstieg?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die 343,11 € mehr sehen dramatischer aus, als sie sind. 2025 enthalten die Heizkosten erstmals die Wartung der Wärmepumpe (562,28 € für die ganze Anlage) und die Abrechnungskosten (260,55 €), die 2024 separat standen oder gar nicht anfielen. Grob gerechnet sind davon rund 175 € Umschichtung — der echte Anstieg liegt eher bei 170 € und damit im Rahmen der Energiepreise.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Vor dem Versenden</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Abrechnungsfrist</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Für 2025 läuft sie am 31.12.2026 ab (§ 556 Abs. 3 BGB). Danach kannst du nichts mehr nachfordern. Da es ein Guthaben ist, droht dir kein Verlust — aber die Herabsetzung der Vorauszahlung willst du rechtzeitig wirksam machen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,55 € ohne nähere Bezeichnung. Beim Verwalter erfragen, was dahinter steckt — ein Mieter darf das wissen wollen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9,63 € sind umlagefähig (§ 2 Nr. 2 BetrKV). Nicht zu verwechseln mit der Miete von Rauchwarnmeldern, die es nicht wäre.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Belegeinsicht</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Du musst sie gewähren, wenn Huber darum bittet. Die Unterlagen der Verwaltung bereithalten.</t>
   </si>
   <si>
     <t xml:space="preserve">Was dich aus der Eigentümerversammlung betrifft</t>
@@ -397,7 +443,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.000"/>
     <numFmt numFmtId="166" formatCode="#,##0.00&quot; €&quot;;\-#,##0.00&quot; €&quot;;\-"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -481,8 +527,16 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="9"/>
+      <color rgb="FFC00000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -510,6 +564,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9E1D9"/>
+        <bgColor rgb="FFE8E8E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4E4"/>
         <bgColor rgb="FFE8E8E8"/>
       </patternFill>
     </fill>
@@ -572,7 +632,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="37">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -682,7 +742,35 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -706,7 +794,7 @@
     <indexedColors>
       <rgbColor rgb="FF000000"/>
       <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FFC00000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -743,7 +831,7 @@
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFFCE4E4"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -1539,13 +1627,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="46"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1682,108 +1769,318 @@
       <c r="A20" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C20" s="27" t="s">
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="27" t="s">
+        <v>11</v>
+      </c>
+      <c r="B21" s="28" t="s">
         <v>73</v>
       </c>
-      <c r="D20" s="27" t="s">
+      <c r="C21" s="28" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
+      <c r="D21" s="28" t="s">
         <v>75</v>
       </c>
-      <c r="C21" s="14" t="n">
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B22" s="14" t="n">
+        <v>212.74</v>
+      </c>
+      <c r="C22" s="14" t="n">
+        <v>219.77</v>
+      </c>
+      <c r="D22" s="14" t="n">
+        <f aca="false">C22-B22</f>
+        <v>7.03</v>
+      </c>
+      <c r="E22" s="23"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="14" t="n">
+        <v>73.95</v>
+      </c>
+      <c r="C23" s="14" t="n">
+        <v>75.91</v>
+      </c>
+      <c r="D23" s="14" t="n">
+        <f aca="false">C23-B23</f>
+        <v>1.95999999999999</v>
+      </c>
+      <c r="E23" s="23"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="14" t="n">
+        <v>20.35</v>
+      </c>
+      <c r="C24" s="14" t="n">
+        <v>7.86</v>
+      </c>
+      <c r="D24" s="14" t="n">
+        <f aca="false">C24-B24</f>
+        <v>-12.49</v>
+      </c>
+      <c r="E24" s="23"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25" s="14" t="n">
+        <v>58.92</v>
+      </c>
+      <c r="C25" s="14" t="n">
+        <v>54.24</v>
+      </c>
+      <c r="D25" s="14" t="n">
+        <f aca="false">C25-B25</f>
+        <v>-4.68</v>
+      </c>
+      <c r="E25" s="23"/>
+    </row>
+    <row r="26" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="30" t="s">
+        <v>76</v>
+      </c>
+      <c r="B26" s="31" t="s">
+        <v>77</v>
+      </c>
+      <c r="C26" s="31"/>
+      <c r="D26" s="31"/>
+      <c r="E26" s="31"/>
+    </row>
+    <row r="27" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="30" t="s">
+        <v>31</v>
+      </c>
+      <c r="B27" s="31" t="s">
+        <v>78</v>
+      </c>
+      <c r="C27" s="31"/>
+      <c r="D27" s="31"/>
+      <c r="E27" s="31"/>
+    </row>
+    <row r="28" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28" s="31" t="s">
+        <v>79</v>
+      </c>
+      <c r="C28" s="31"/>
+      <c r="D28" s="31"/>
+      <c r="E28" s="31"/>
+    </row>
+    <row r="29" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="30" t="s">
+        <v>80</v>
+      </c>
+      <c r="B29" s="31" t="s">
+        <v>81</v>
+      </c>
+      <c r="C29" s="31"/>
+      <c r="D29" s="31"/>
+      <c r="E29" s="31"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="14" t="n">
+        <v>9.63</v>
+      </c>
+      <c r="D30" s="14" t="n">
+        <f aca="false">C30-B30</f>
+        <v>9.63</v>
+      </c>
+      <c r="E30" s="23" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B31" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="14" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="D31" s="14" t="n">
+        <f aca="false">C31-B31</f>
+        <v>2.55</v>
+      </c>
+      <c r="E31" s="23" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="B32" s="14" t="n">
+        <v>93.96</v>
+      </c>
+      <c r="C32" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="14" t="n">
+        <f aca="false">C32-B32</f>
+        <v>-93.96</v>
+      </c>
+      <c r="E32" s="23" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="B33" s="14" t="n">
+        <v>37.24</v>
+      </c>
+      <c r="C33" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="14" t="n">
+        <f aca="false">C33-B33</f>
+        <v>-37.24</v>
+      </c>
+      <c r="E33" s="23" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="32" t="s">
+        <v>89</v>
+      </c>
+      <c r="B34" s="33" t="n">
+        <v>52.7</v>
+      </c>
+      <c r="C34" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="33" t="n">
+        <f aca="false">C34-B34</f>
+        <v>-52.7</v>
+      </c>
+      <c r="E34" s="34" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="B35" s="33" t="n">
+        <v>8.73</v>
+      </c>
+      <c r="C35" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="33" t="n">
+        <f aca="false">C35-B35</f>
+        <v>-8.73</v>
+      </c>
+      <c r="E35" s="34" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="B36" s="16" t="n">
+        <v>821.49</v>
+      </c>
+      <c r="C36" s="16" t="n">
+        <v>692.65</v>
+      </c>
+      <c r="D36" s="16" t="n">
+        <f aca="false">C36-B36</f>
+        <v>-128.84</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="15" t="s">
+        <v>93</v>
+      </c>
+      <c r="B37" s="16" t="n">
+        <v>969.75</v>
+      </c>
+      <c r="C37" s="16" t="n">
+        <v>1312.86</v>
+      </c>
+      <c r="D37" s="16" t="n">
+        <f aca="false">C37-B37</f>
+        <v>343.11</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="B38" s="16" t="n">
         <v>1791.24</v>
       </c>
-      <c r="D21" s="14" t="n">
+      <c r="C38" s="16" t="n">
         <v>2005.51</v>
       </c>
-      <c r="E21" s="26" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C22" s="14" t="n">
-        <v>969.75</v>
-      </c>
-      <c r="D22" s="14" t="n">
-        <v>1312.86</v>
-      </c>
-      <c r="E22" s="26"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C23" s="14" t="n">
-        <v>93.96</v>
-      </c>
-      <c r="D23" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="26"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="1" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="28" t="s">
-        <v>80</v>
-      </c>
-      <c r="B26" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7"/>
-    </row>
-    <row r="27" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="28" t="s">
-        <v>31</v>
-      </c>
-      <c r="B27" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="C27" s="7"/>
-      <c r="D27" s="7"/>
-      <c r="E27" s="7"/>
-    </row>
-    <row r="28" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="28" t="s">
-        <v>28</v>
-      </c>
-      <c r="B28" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="C28" s="7"/>
-      <c r="D28" s="7"/>
-      <c r="E28" s="7"/>
-    </row>
-    <row r="29" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="28" t="s">
-        <v>84</v>
-      </c>
-      <c r="B29" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="C29" s="7"/>
-      <c r="D29" s="7"/>
-      <c r="E29" s="7"/>
+      <c r="D38" s="16" t="n">
+        <f aca="false">C38-B38</f>
+        <v>214.27</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="C40" s="7"/>
+      <c r="D40" s="7"/>
+      <c r="E40" s="7"/>
+    </row>
+    <row r="42" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="C42" s="7"/>
+      <c r="D42" s="7"/>
+      <c r="E42" s="7"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="0" t="s">
+        <v>99</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="E10:E13"/>
-    <mergeCell ref="E21:E23"/>
     <mergeCell ref="B26:E26"/>
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="B28:E28"/>
     <mergeCell ref="B29:E29"/>
+    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="B42:E42"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1809,76 +2106,76 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="22" t="s">
-        <v>86</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="23" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="B4" s="29" t="s">
-        <v>89</v>
+      <c r="A4" s="35" t="s">
+        <v>102</v>
+      </c>
+      <c r="B4" s="36" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="28" t="s">
-        <v>90</v>
-      </c>
-      <c r="B5" s="29" t="s">
-        <v>91</v>
+      <c r="A5" s="35" t="s">
+        <v>104</v>
+      </c>
+      <c r="B5" s="36" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="28" t="s">
-        <v>92</v>
-      </c>
-      <c r="B6" s="29" t="s">
-        <v>93</v>
+      <c r="A6" s="35" t="s">
+        <v>106</v>
+      </c>
+      <c r="B6" s="36" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="28" t="s">
-        <v>94</v>
-      </c>
-      <c r="B7" s="29" t="s">
-        <v>95</v>
+      <c r="A7" s="35" t="s">
+        <v>108</v>
+      </c>
+      <c r="B7" s="36" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="28" t="s">
-        <v>96</v>
-      </c>
-      <c r="B8" s="29" t="s">
-        <v>97</v>
+      <c r="A8" s="35" t="s">
+        <v>110</v>
+      </c>
+      <c r="B8" s="36" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="28" t="s">
-        <v>98</v>
-      </c>
-      <c r="B9" s="29" t="s">
-        <v>99</v>
+      <c r="A9" s="35" t="s">
+        <v>112</v>
+      </c>
+      <c r="B9" s="36" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="28" t="s">
-        <v>100</v>
-      </c>
-      <c r="B10" s="29" t="s">
-        <v>101</v>
+      <c r="A10" s="35" t="s">
+        <v>114</v>
+      </c>
+      <c r="B10" s="36" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="28" t="s">
-        <v>102</v>
-      </c>
-      <c r="B11" s="29" t="s">
-        <v>103</v>
+      <c r="A11" s="35" t="s">
+        <v>116</v>
+      </c>
+      <c r="B11" s="36" t="s">
+        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>